<commit_message>
update to be generic on sample/profile
</commit_message>
<xml_diff>
--- a/SimpleCSV/SoilTemplate.xlsx
+++ b/SimpleCSV/SoilTemplate.xlsx
@@ -1,21 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29523"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Kathi\Dropbox\cove\SoilWise\WP2\CelineExamples\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\projects\soilwise\soil-observation-data-encodings\SimpleCSV\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0DF92B52-7406-47BC-8DEF-DBFD216738FD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{35A50D01-6954-4B89-9CAA-DEE52E0E900F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" firstSheet="1" activeTab="1" xr2:uid="{9DCE1E4B-6CD1-46B5-8D2E-1D2FE5DA7756}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{9DCE1E4B-6CD1-46B5-8D2E-1D2FE5DA7756}"/>
   </bookViews>
   <sheets>
-    <sheet name="ReadMe" sheetId="4" r:id="rId1"/>
+    <sheet name="Metadata" sheetId="4" r:id="rId1"/>
     <sheet name="ObservableProperties" sheetId="1" r:id="rId2"/>
-    <sheet name="SpatialObjects" sheetId="2" r:id="rId3"/>
+    <sheet name="Samples" sheetId="2" r:id="rId3"/>
     <sheet name="Data" sheetId="3" r:id="rId4"/>
   </sheets>
   <calcPr calcId="191028"/>
@@ -39,29 +39,17 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="104" uniqueCount="63">
-  <si>
-    <t xml:space="preserve">Project: </t>
-  </si>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="100" uniqueCount="64">
   <si>
     <t>SoilWise Template</t>
   </si>
   <si>
-    <t>Publication:</t>
-  </si>
-  <si>
-    <t>Dummy Publication</t>
-  </si>
-  <si>
     <t>Funding</t>
   </si>
   <si>
     <t>XXX</t>
   </si>
   <si>
-    <t>Experiment:</t>
-  </si>
-  <si>
     <t>Dummy data</t>
   </si>
   <si>
@@ -74,33 +62,18 @@
     <t>Country:</t>
   </si>
   <si>
-    <t xml:space="preserve">Sampling: </t>
-  </si>
-  <si>
-    <t>8 plots</t>
-  </si>
-  <si>
     <t>Date</t>
   </si>
   <si>
-    <t>2020 - 2022</t>
-  </si>
-  <si>
     <t>CRS:</t>
   </si>
   <si>
     <t>EPSG:4326</t>
   </si>
   <si>
-    <t>Mandatory</t>
-  </si>
-  <si>
     <t>Variable</t>
   </si>
   <si>
-    <t>Description</t>
-  </si>
-  <si>
     <t>Variable URI</t>
   </si>
   <si>
@@ -113,9 +86,6 @@
     <t>Methodology URI</t>
   </si>
   <si>
-    <t>Sample Preparation</t>
-  </si>
-  <si>
     <t>GI</t>
   </si>
   <si>
@@ -126,9 +96,6 @@
   </si>
   <si>
     <t>Proportion of green pixels in photographs</t>
-  </si>
-  <si>
-    <t>Soil DW</t>
   </si>
   <si>
     <t>C</t>
@@ -192,27 +159,12 @@
     <t xml:space="preserve">Waithaisong et al., 2020 </t>
   </si>
   <si>
-    <t>Plot</t>
-  </si>
-  <si>
-    <t>x</t>
-  </si>
-  <si>
-    <t>y</t>
-  </si>
-  <si>
-    <t>Accuracy</t>
-  </si>
-  <si>
     <t>Upper Depth Layer</t>
   </si>
   <si>
     <t>Lower Depth Layer</t>
   </si>
   <si>
-    <t>Object Type</t>
-  </si>
-  <si>
     <t>Unterpullendorf</t>
   </si>
   <si>
@@ -241,6 +193,57 @@
   </si>
   <si>
     <t>POlsen</t>
+  </si>
+  <si>
+    <t>Period:</t>
+  </si>
+  <si>
+    <t>License:</t>
+  </si>
+  <si>
+    <t>CC-BY</t>
+  </si>
+  <si>
+    <t>Author:</t>
+  </si>
+  <si>
+    <t>Kathi Schleidt</t>
+  </si>
+  <si>
+    <t>2022 - 2024</t>
+  </si>
+  <si>
+    <t>Abstract:</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Title: </t>
+  </si>
+  <si>
+    <t>Identification</t>
+  </si>
+  <si>
+    <t>https://doi.org/10.5432/aazzbb</t>
+  </si>
+  <si>
+    <t>Identification:</t>
+  </si>
+  <si>
+    <t>X</t>
+  </si>
+  <si>
+    <t>Y</t>
+  </si>
+  <si>
+    <t>Feature of Interest</t>
+  </si>
+  <si>
+    <t>Column name</t>
+  </si>
+  <si>
+    <t>Unit URI</t>
+  </si>
+  <si>
+    <t>SampleID</t>
   </si>
 </sst>
 </file>
@@ -250,7 +253,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.000"/>
   </numFmts>
-  <fonts count="6">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -350,7 +353,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
@@ -366,9 +369,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -379,14 +379,14 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="2">
-    <cellStyle name="Collegamento ipertestuale" xfId="1" builtinId="8"/>
-    <cellStyle name="Normale" xfId="0" builtinId="0"/>
+    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -402,9 +402,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -442,7 +442,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -548,7 +548,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -690,7 +690,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -699,92 +699,97 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{85928423-BA79-402A-98D3-266C23F871FF}">
   <dimension ref="A1:C10"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="14.28515625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="97.7109375" customWidth="1"/>
+    <col min="1" max="1" width="14.33203125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="97.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="15.75">
+    <row r="1" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="B1" s="11" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A2" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="B2" s="6" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="6" t="s">
+    </row>
+    <row r="3" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A3" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="B3" s="6" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A4" s="1" t="s">
         <v>1</v>
       </c>
-    </row>
-    <row r="2" spans="1:3" ht="15.75">
-      <c r="A2" s="1" t="s">
+      <c r="B4" s="6" t="s">
         <v>2</v>
       </c>
-      <c r="B2" s="7" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" ht="15.75">
-      <c r="A3" s="1" t="s">
+    </row>
+    <row r="5" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A5" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B3" s="6" t="s">
+      <c r="B5" s="6" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="4" spans="1:3" ht="15.75">
-      <c r="A4" s="1" t="s">
+    <row r="6" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A6" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="B4" s="6" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3" ht="15.75">
-      <c r="A5" s="1" t="s">
+      <c r="B6" s="6" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A7" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="B7" s="6" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A8" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="B5" s="6" t="s">
+      <c r="B8" s="14" t="s">
         <v>9</v>
       </c>
-    </row>
-    <row r="6" spans="1:3" ht="15.75">
-      <c r="A6" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="B6" s="6" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3" ht="15.75">
-      <c r="A7" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="B7" s="6" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="8" spans="1:3" ht="15.75">
-      <c r="A8" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="B8" s="6" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="9" spans="1:3" ht="15.75">
+      <c r="C8" s="13"/>
+    </row>
+    <row r="9" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A9" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="B9" s="14" t="s">
-        <v>16</v>
-      </c>
-      <c r="C9" s="15" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="10" spans="1:3">
-      <c r="A10" s="6"/>
-      <c r="B10" s="6"/>
+        <v>48</v>
+      </c>
+      <c r="B9" s="6" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A10" s="7" t="s">
+        <v>50</v>
+      </c>
+      <c r="B10" s="6" t="s">
+        <v>51</v>
+      </c>
     </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink ref="B1" r:id="rId1" xr:uid="{33739310-5776-4BDA-9103-DF7D7CF23DC2}"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
@@ -792,125 +797,117 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8C509145-F6A6-492C-969F-82100225473C}">
   <dimension ref="A1:G5"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="15.5703125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="24.5703125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="71.28515625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="16.140625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="38.85546875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="38.85546875" customWidth="1"/>
-    <col min="7" max="7" width="20.7109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="15.5546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="24.5546875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="71.33203125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="16.109375" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="16.109375" customWidth="1"/>
+    <col min="6" max="6" width="38.88671875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="38.88671875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" ht="15.75">
+    <row r="1" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
-        <v>18</v>
+        <v>61</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>19</v>
+        <v>10</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>20</v>
+        <v>11</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>21</v>
+        <v>12</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>22</v>
+        <v>62</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="G1" s="8" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="2" spans="1:7">
+        <v>13</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
-        <v>25</v>
+        <v>15</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>26</v>
+        <v>16</v>
       </c>
       <c r="C2" s="2"/>
       <c r="D2" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="E2" s="2"/>
+      <c r="F2" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="G2" s="10"/>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A3" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="C3" s="11" t="s">
+        <v>21</v>
+      </c>
+      <c r="D3" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="E3" s="2"/>
+      <c r="F3" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="G3" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A4" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="C4" s="12" t="s">
         <v>27</v>
       </c>
-      <c r="E2" s="2" t="s">
+      <c r="D4" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="E4" s="2"/>
+      <c r="F4" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="F2" s="11"/>
-      <c r="G2" s="11" t="s">
+      <c r="G4" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="3" spans="1:7">
-      <c r="A3" s="2" t="s">
+    <row r="5" spans="1:7" ht="16.2" x14ac:dyDescent="0.3">
+      <c r="A5" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="B3" s="2" t="s">
+      <c r="B5" s="2" t="s">
         <v>31</v>
       </c>
-      <c r="C3" s="12" t="s">
+      <c r="C5" s="12" t="s">
         <v>32</v>
       </c>
-      <c r="D3" s="2" t="s">
+      <c r="D5" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="E3" s="2" t="s">
+      <c r="E5" s="2"/>
+      <c r="F5" s="2" t="s">
         <v>34</v>
       </c>
-      <c r="F3" t="s">
-        <v>35</v>
-      </c>
-      <c r="G3" s="11" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="4" spans="1:7">
-      <c r="A4" s="2" t="s">
-        <v>36</v>
-      </c>
-      <c r="B4" s="2" t="s">
-        <v>37</v>
-      </c>
-      <c r="C4" s="13" t="s">
-        <v>38</v>
-      </c>
-      <c r="D4" s="2" t="s">
-        <v>33</v>
-      </c>
-      <c r="E4" s="2" t="s">
-        <v>39</v>
-      </c>
-      <c r="F4" t="s">
-        <v>40</v>
-      </c>
-      <c r="G4" s="11" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="5" spans="1:7" ht="17.25">
-      <c r="A5" s="2" t="s">
-        <v>41</v>
-      </c>
-      <c r="B5" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="C5" s="13" t="s">
-        <v>43</v>
-      </c>
-      <c r="D5" s="2" t="s">
-        <v>44</v>
-      </c>
-      <c r="E5" s="2" t="s">
-        <v>45</v>
-      </c>
-      <c r="F5" s="11"/>
-      <c r="G5" s="11" t="s">
-        <v>29</v>
-      </c>
+      <c r="G5" s="10"/>
     </row>
   </sheetData>
   <hyperlinks>
@@ -919,47 +916,45 @@
     <hyperlink ref="C5" r:id="rId3" xr:uid="{1EC27527-3F9C-465E-BDA3-D5CF5C93B31C}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="0" verticalDpi="0" r:id="rId4"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8818055C-AB83-43A8-BE9A-02F4FE494E8D}">
-  <dimension ref="A1:G9"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <dimension ref="A1:F9"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="20.7109375" style="3" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="20.6640625" style="3" bestFit="1" customWidth="1"/>
     <col min="2" max="3" width="6" style="3" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="9.85546875" bestFit="1" customWidth="1"/>
-    <col min="5" max="6" width="19.7109375" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="12.7109375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="6.6640625" customWidth="1"/>
+    <col min="5" max="5" width="6.44140625" customWidth="1"/>
+    <col min="6" max="6" width="20.21875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" ht="15.75">
+    <row r="1" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
-        <v>46</v>
+        <v>55</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>47</v>
+        <v>58</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>48</v>
-      </c>
-      <c r="D1" s="8" t="s">
-        <v>49</v>
-      </c>
-      <c r="E1" s="8" t="s">
-        <v>50</v>
-      </c>
-      <c r="F1" s="8" t="s">
-        <v>51</v>
-      </c>
-      <c r="G1" s="8" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="2" spans="1:7">
-      <c r="A2" s="9" t="s">
-        <v>53</v>
+        <v>59</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A2" s="8" t="s">
+        <v>37</v>
       </c>
       <c r="B2" s="3">
         <v>47.49</v>
@@ -967,19 +962,19 @@
       <c r="C2" s="3">
         <v>16.559999999999999</v>
       </c>
+      <c r="D2">
+        <v>10</v>
+      </c>
       <c r="E2">
-        <v>10</v>
-      </c>
-      <c r="F2">
         <v>20</v>
       </c>
-      <c r="G2" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="3" spans="1:7">
-      <c r="A3" s="9" t="s">
-        <v>55</v>
+      <c r="F2" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A3" s="8" t="s">
+        <v>39</v>
       </c>
       <c r="B3" s="3">
         <v>48.12</v>
@@ -987,19 +982,19 @@
       <c r="C3" s="3">
         <v>16.05</v>
       </c>
+      <c r="D3">
+        <v>10</v>
+      </c>
       <c r="E3">
-        <v>10</v>
-      </c>
-      <c r="F3">
         <v>20</v>
       </c>
-      <c r="G3" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="4" spans="1:7">
-      <c r="A4" s="9" t="s">
-        <v>56</v>
+      <c r="F3" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A4" s="8" t="s">
+        <v>40</v>
       </c>
       <c r="B4" s="3">
         <v>47.88</v>
@@ -1007,19 +1002,19 @@
       <c r="C4" s="3">
         <v>13.35</v>
       </c>
+      <c r="D4">
+        <v>10</v>
+      </c>
       <c r="E4">
-        <v>10</v>
-      </c>
-      <c r="F4">
         <v>20</v>
       </c>
-      <c r="G4" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="5" spans="1:7">
-      <c r="A5" s="9" t="s">
-        <v>57</v>
+      <c r="F4" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A5" s="8" t="s">
+        <v>41</v>
       </c>
       <c r="B5" s="3">
         <v>47.63</v>
@@ -1027,19 +1022,19 @@
       <c r="C5" s="3">
         <v>15.66</v>
       </c>
+      <c r="D5">
+        <v>10</v>
+      </c>
       <c r="E5">
-        <v>10</v>
-      </c>
-      <c r="F5">
         <v>20</v>
       </c>
-      <c r="G5" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="6" spans="1:7">
-      <c r="A6" s="9" t="s">
-        <v>58</v>
+      <c r="F5" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A6" s="8" t="s">
+        <v>42</v>
       </c>
       <c r="B6" s="3">
         <v>47.06</v>
@@ -1047,19 +1042,19 @@
       <c r="C6" s="3">
         <v>14.11</v>
       </c>
+      <c r="D6">
+        <v>10</v>
+      </c>
       <c r="E6">
-        <v>10</v>
-      </c>
-      <c r="F6">
         <v>20</v>
       </c>
-      <c r="G6" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="7" spans="1:7">
-      <c r="A7" s="9" t="s">
-        <v>59</v>
+      <c r="F6" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A7" s="8" t="s">
+        <v>43</v>
       </c>
       <c r="B7" s="3">
         <v>47.33</v>
@@ -1067,19 +1062,19 @@
       <c r="C7" s="3">
         <v>12.41</v>
       </c>
+      <c r="D7">
+        <v>10</v>
+      </c>
       <c r="E7">
-        <v>10</v>
-      </c>
-      <c r="F7">
         <v>20</v>
       </c>
-      <c r="G7" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="8" spans="1:7">
-      <c r="A8" s="9" t="s">
-        <v>60</v>
+      <c r="F7" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A8" s="8" t="s">
+        <v>44</v>
       </c>
       <c r="B8" s="3">
         <v>47.84</v>
@@ -1087,19 +1082,19 @@
       <c r="C8" s="3">
         <v>14.44</v>
       </c>
+      <c r="D8">
+        <v>10</v>
+      </c>
       <c r="E8">
-        <v>10</v>
-      </c>
-      <c r="F8">
         <v>20</v>
       </c>
-      <c r="G8" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="9" spans="1:7">
-      <c r="A9" s="9" t="s">
-        <v>61</v>
+      <c r="F8" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A9" s="8" t="s">
+        <v>45</v>
       </c>
       <c r="B9" s="3">
         <v>47.84</v>
@@ -1107,55 +1102,56 @@
       <c r="C9" s="3">
         <v>14.44</v>
       </c>
+      <c r="D9">
+        <v>20</v>
+      </c>
       <c r="E9">
-        <v>10</v>
-      </c>
-      <c r="F9">
-        <v>20</v>
-      </c>
-      <c r="G9" t="s">
-        <v>54</v>
+        <v>40</v>
+      </c>
+      <c r="F9" t="s">
+        <v>38</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="0" verticalDpi="0" r:id="rId1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3F9B60B5-15F3-4C2F-BF4C-90A521C6DDDC}">
   <dimension ref="A1:G52"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="20.7109375" style="3" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="10.85546875" style="3" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="9.140625" style="4"/>
-    <col min="4" max="6" width="9.140625" style="5"/>
+    <col min="1" max="1" width="20.6640625" style="3" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.88671875" style="3" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="9.109375" style="4"/>
+    <col min="4" max="6" width="9.109375" style="5"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" ht="15.75">
+    <row r="1" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="F1" s="1" t="s">
         <v>46</v>
       </c>
-      <c r="B1" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>25</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>30</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>36</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>62</v>
-      </c>
-    </row>
-    <row r="2" spans="1:7">
-      <c r="A2" s="9" t="s">
-        <v>53</v>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A2" s="8" t="s">
+        <v>37</v>
       </c>
       <c r="B2" s="6">
         <v>2020</v>
@@ -1174,9 +1170,9 @@
       </c>
       <c r="G2" s="5"/>
     </row>
-    <row r="3" spans="1:7">
-      <c r="A3" s="9" t="s">
-        <v>55</v>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A3" s="8" t="s">
+        <v>39</v>
       </c>
       <c r="B3" s="6">
         <v>2020</v>
@@ -1195,9 +1191,9 @@
       </c>
       <c r="G3" s="5"/>
     </row>
-    <row r="4" spans="1:7">
-      <c r="A4" s="9" t="s">
-        <v>56</v>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A4" s="8" t="s">
+        <v>40</v>
       </c>
       <c r="B4" s="6">
         <v>2020</v>
@@ -1216,9 +1212,9 @@
       </c>
       <c r="G4" s="5"/>
     </row>
-    <row r="5" spans="1:7">
-      <c r="A5" s="9" t="s">
-        <v>57</v>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A5" s="8" t="s">
+        <v>41</v>
       </c>
       <c r="B5" s="6">
         <v>2020</v>
@@ -1237,9 +1233,9 @@
       </c>
       <c r="G5" s="5"/>
     </row>
-    <row r="6" spans="1:7">
-      <c r="A6" s="9" t="s">
-        <v>58</v>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A6" s="8" t="s">
+        <v>42</v>
       </c>
       <c r="B6" s="6">
         <v>2020</v>
@@ -1258,9 +1254,9 @@
       </c>
       <c r="G6" s="5"/>
     </row>
-    <row r="7" spans="1:7">
-      <c r="A7" s="9" t="s">
-        <v>59</v>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A7" s="8" t="s">
+        <v>43</v>
       </c>
       <c r="B7" s="6">
         <v>2020</v>
@@ -1279,9 +1275,9 @@
       </c>
       <c r="G7" s="5"/>
     </row>
-    <row r="8" spans="1:7">
-      <c r="A8" s="9" t="s">
-        <v>60</v>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A8" s="8" t="s">
+        <v>44</v>
       </c>
       <c r="B8" s="6">
         <v>2020</v>
@@ -1300,9 +1296,9 @@
       </c>
       <c r="G8" s="5"/>
     </row>
-    <row r="9" spans="1:7">
-      <c r="A9" s="9" t="s">
-        <v>61</v>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A9" s="8" t="s">
+        <v>45</v>
       </c>
       <c r="B9" s="6">
         <v>2020</v>
@@ -1321,11 +1317,11 @@
       </c>
       <c r="G9" s="5"/>
     </row>
-    <row r="10" spans="1:7">
-      <c r="A10" s="9" t="s">
-        <v>53</v>
-      </c>
-      <c r="B10" s="10">
+    <row r="10" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A10" s="8" t="s">
+        <v>37</v>
+      </c>
+      <c r="B10" s="9">
         <v>44259</v>
       </c>
       <c r="C10" s="4">
@@ -1342,11 +1338,11 @@
       </c>
       <c r="G10" s="5"/>
     </row>
-    <row r="11" spans="1:7">
-      <c r="A11" s="9" t="s">
-        <v>55</v>
-      </c>
-      <c r="B11" s="10">
+    <row r="11" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A11" s="8" t="s">
+        <v>39</v>
+      </c>
+      <c r="B11" s="9">
         <v>44260</v>
       </c>
       <c r="C11" s="4">
@@ -1363,11 +1359,11 @@
       </c>
       <c r="G11" s="5"/>
     </row>
-    <row r="12" spans="1:7">
-      <c r="A12" s="9" t="s">
-        <v>56</v>
-      </c>
-      <c r="B12" s="10">
+    <row r="12" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A12" s="8" t="s">
+        <v>40</v>
+      </c>
+      <c r="B12" s="9">
         <v>44261</v>
       </c>
       <c r="C12" s="4">
@@ -1384,11 +1380,11 @@
       </c>
       <c r="G12" s="5"/>
     </row>
-    <row r="13" spans="1:7">
-      <c r="A13" s="9" t="s">
-        <v>57</v>
-      </c>
-      <c r="B13" s="10">
+    <row r="13" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A13" s="8" t="s">
+        <v>41</v>
+      </c>
+      <c r="B13" s="9">
         <v>44262</v>
       </c>
       <c r="C13" s="4">
@@ -1405,11 +1401,11 @@
       </c>
       <c r="G13" s="5"/>
     </row>
-    <row r="14" spans="1:7">
-      <c r="A14" s="9" t="s">
-        <v>58</v>
-      </c>
-      <c r="B14" s="10">
+    <row r="14" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A14" s="8" t="s">
+        <v>42</v>
+      </c>
+      <c r="B14" s="9">
         <v>44263</v>
       </c>
       <c r="C14" s="4">
@@ -1426,11 +1422,11 @@
       </c>
       <c r="G14" s="5"/>
     </row>
-    <row r="15" spans="1:7">
-      <c r="A15" s="9" t="s">
-        <v>59</v>
-      </c>
-      <c r="B15" s="10">
+    <row r="15" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A15" s="8" t="s">
+        <v>43</v>
+      </c>
+      <c r="B15" s="9">
         <v>44264</v>
       </c>
       <c r="C15" s="4">
@@ -1447,11 +1443,11 @@
       </c>
       <c r="G15" s="5"/>
     </row>
-    <row r="16" spans="1:7">
-      <c r="A16" s="9" t="s">
-        <v>60</v>
-      </c>
-      <c r="B16" s="10">
+    <row r="16" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A16" s="8" t="s">
+        <v>44</v>
+      </c>
+      <c r="B16" s="9">
         <v>44265</v>
       </c>
       <c r="C16" s="4">
@@ -1468,11 +1464,11 @@
       </c>
       <c r="G16" s="5"/>
     </row>
-    <row r="17" spans="1:7">
-      <c r="A17" s="9" t="s">
-        <v>61</v>
-      </c>
-      <c r="B17" s="10">
+    <row r="17" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A17" s="8" t="s">
+        <v>45</v>
+      </c>
+      <c r="B17" s="9">
         <v>44266</v>
       </c>
       <c r="C17" s="4">
@@ -1489,11 +1485,11 @@
       </c>
       <c r="G17" s="5"/>
     </row>
-    <row r="18" spans="1:7">
-      <c r="A18" s="9" t="s">
-        <v>53</v>
-      </c>
-      <c r="B18" s="10">
+    <row r="18" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A18" s="8" t="s">
+        <v>37</v>
+      </c>
+      <c r="B18" s="9">
         <v>44656</v>
       </c>
       <c r="C18" s="4">
@@ -1510,11 +1506,11 @@
       </c>
       <c r="G18" s="5"/>
     </row>
-    <row r="19" spans="1:7">
-      <c r="A19" s="9" t="s">
-        <v>55</v>
-      </c>
-      <c r="B19" s="10">
+    <row r="19" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A19" s="8" t="s">
+        <v>39</v>
+      </c>
+      <c r="B19" s="9">
         <v>44657</v>
       </c>
       <c r="C19" s="4">
@@ -1531,11 +1527,11 @@
       </c>
       <c r="G19" s="5"/>
     </row>
-    <row r="20" spans="1:7">
-      <c r="A20" s="9" t="s">
-        <v>56</v>
-      </c>
-      <c r="B20" s="10">
+    <row r="20" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A20" s="8" t="s">
+        <v>40</v>
+      </c>
+      <c r="B20" s="9">
         <v>44658</v>
       </c>
       <c r="C20" s="4">
@@ -1552,11 +1548,11 @@
       </c>
       <c r="G20" s="5"/>
     </row>
-    <row r="21" spans="1:7">
-      <c r="A21" s="9" t="s">
-        <v>57</v>
-      </c>
-      <c r="B21" s="10">
+    <row r="21" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A21" s="8" t="s">
+        <v>41</v>
+      </c>
+      <c r="B21" s="9">
         <v>44659</v>
       </c>
       <c r="C21" s="4">
@@ -1573,11 +1569,11 @@
       </c>
       <c r="G21" s="5"/>
     </row>
-    <row r="22" spans="1:7">
-      <c r="A22" s="9" t="s">
-        <v>58</v>
-      </c>
-      <c r="B22" s="10">
+    <row r="22" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A22" s="8" t="s">
+        <v>42</v>
+      </c>
+      <c r="B22" s="9">
         <v>44660</v>
       </c>
       <c r="C22" s="4">
@@ -1594,11 +1590,11 @@
       </c>
       <c r="G22" s="5"/>
     </row>
-    <row r="23" spans="1:7">
-      <c r="A23" s="9" t="s">
-        <v>59</v>
-      </c>
-      <c r="B23" s="10">
+    <row r="23" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A23" s="8" t="s">
+        <v>43</v>
+      </c>
+      <c r="B23" s="9">
         <v>44661</v>
       </c>
       <c r="C23" s="4">
@@ -1615,11 +1611,11 @@
       </c>
       <c r="G23" s="5"/>
     </row>
-    <row r="24" spans="1:7">
-      <c r="A24" s="9" t="s">
-        <v>60</v>
-      </c>
-      <c r="B24" s="10">
+    <row r="24" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A24" s="8" t="s">
+        <v>44</v>
+      </c>
+      <c r="B24" s="9">
         <v>44662</v>
       </c>
       <c r="C24" s="4">
@@ -1636,11 +1632,11 @@
       </c>
       <c r="G24" s="5"/>
     </row>
-    <row r="25" spans="1:7">
-      <c r="A25" s="9" t="s">
-        <v>61</v>
-      </c>
-      <c r="B25" s="10">
+    <row r="25" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A25" s="8" t="s">
+        <v>45</v>
+      </c>
+      <c r="B25" s="9">
         <v>44663</v>
       </c>
       <c r="C25" s="4">
@@ -1657,89 +1653,90 @@
       </c>
       <c r="G25" s="5"/>
     </row>
-    <row r="26" spans="1:7">
+    <row r="26" spans="1:7" x14ac:dyDescent="0.3">
       <c r="B26" s="6"/>
     </row>
-    <row r="27" spans="1:7">
+    <row r="27" spans="1:7" x14ac:dyDescent="0.3">
       <c r="B27" s="6"/>
     </row>
-    <row r="28" spans="1:7">
+    <row r="28" spans="1:7" x14ac:dyDescent="0.3">
       <c r="B28" s="6"/>
     </row>
-    <row r="29" spans="1:7">
+    <row r="29" spans="1:7" x14ac:dyDescent="0.3">
       <c r="B29" s="6"/>
     </row>
-    <row r="30" spans="1:7">
+    <row r="30" spans="1:7" x14ac:dyDescent="0.3">
       <c r="B30" s="6"/>
     </row>
-    <row r="31" spans="1:7">
+    <row r="31" spans="1:7" x14ac:dyDescent="0.3">
       <c r="B31" s="6"/>
     </row>
-    <row r="32" spans="1:7">
+    <row r="32" spans="1:7" x14ac:dyDescent="0.3">
       <c r="B32" s="6"/>
     </row>
-    <row r="33" spans="2:2">
+    <row r="33" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B33" s="6"/>
     </row>
-    <row r="34" spans="2:2">
+    <row r="34" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B34" s="6"/>
     </row>
-    <row r="35" spans="2:2">
+    <row r="35" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B35" s="6"/>
     </row>
-    <row r="36" spans="2:2">
+    <row r="36" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B36" s="6"/>
     </row>
-    <row r="37" spans="2:2">
+    <row r="37" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B37" s="6"/>
     </row>
-    <row r="38" spans="2:2">
+    <row r="38" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B38" s="6"/>
     </row>
-    <row r="39" spans="2:2">
+    <row r="39" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B39" s="6"/>
     </row>
-    <row r="40" spans="2:2">
+    <row r="40" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B40" s="6"/>
     </row>
-    <row r="41" spans="2:2">
+    <row r="41" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B41" s="6"/>
     </row>
-    <row r="42" spans="2:2">
+    <row r="42" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B42" s="6"/>
     </row>
-    <row r="43" spans="2:2">
+    <row r="43" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B43" s="6"/>
     </row>
-    <row r="44" spans="2:2">
+    <row r="44" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B44" s="6"/>
     </row>
-    <row r="45" spans="2:2">
+    <row r="45" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B45" s="6"/>
     </row>
-    <row r="46" spans="2:2">
+    <row r="46" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B46" s="6"/>
     </row>
-    <row r="47" spans="2:2">
+    <row r="47" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B47" s="6"/>
     </row>
-    <row r="48" spans="2:2">
+    <row r="48" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B48" s="6"/>
     </row>
-    <row r="49" spans="2:2">
+    <row r="49" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B49" s="6"/>
     </row>
-    <row r="50" spans="2:2">
+    <row r="50" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B50" s="6"/>
     </row>
-    <row r="51" spans="2:2">
+    <row r="51" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B51" s="6"/>
     </row>
-    <row r="52" spans="2:2">
+    <row r="52" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B52" s="6"/>
     </row>
   </sheetData>
   <phoneticPr fontId="4" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="0" verticalDpi="0" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>